<commit_message>
feat: implement 5-pillar industry standard upgrades (audio reader, spoiler shield, dynamic OG cards, PWA & offline mode)
</commit_message>
<xml_diff>
--- a/WhereWasI_Comprehensive_E2E_Test_Report.xlsx
+++ b/WhereWasI_Comprehensive_E2E_Test_Report.xlsx
@@ -679,7 +679,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Executed on: 2026-10-05T07:47:20.897Z | Target Environment: http://localhost:3005</t>
+          <t>Executed on: 2026-10-19T19:38:51.275Z | Target Environment: http://localhost:3005</t>
         </is>
       </c>
     </row>
@@ -801,7 +801,7 @@
       </c>
       <c r="H11" s="16" t="inlineStr">
         <is>
-          <t>33 ms</t>
+          <t>2446 ms</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       </c>
       <c r="H12" s="18" t="inlineStr">
         <is>
-          <t>26 ms</t>
+          <t>3262 ms</t>
         </is>
       </c>
     </row>
@@ -859,7 +859,7 @@
       </c>
       <c r="H13" s="16" t="inlineStr">
         <is>
-          <t>33 ms</t>
+          <t>2453 ms</t>
         </is>
       </c>
     </row>
@@ -888,7 +888,7 @@
       </c>
       <c r="H14" s="18" t="inlineStr">
         <is>
-          <t>23 ms</t>
+          <t>3268 ms</t>
         </is>
       </c>
     </row>
@@ -917,7 +917,7 @@
       </c>
       <c r="H15" s="16" t="inlineStr">
         <is>
-          <t>38 ms</t>
+          <t>3257 ms</t>
         </is>
       </c>
     </row>
@@ -946,7 +946,7 @@
       </c>
       <c r="H16" s="18" t="inlineStr">
         <is>
-          <t>7 ms</t>
+          <t>5 ms</t>
         </is>
       </c>
     </row>
@@ -975,7 +975,7 @@
       </c>
       <c r="H17" s="16" t="inlineStr">
         <is>
-          <t>119 ms</t>
+          <t>3453 ms</t>
         </is>
       </c>
     </row>
@@ -1004,7 +1004,7 @@
       </c>
       <c r="H18" s="18" t="inlineStr">
         <is>
-          <t>39 ms</t>
+          <t>3242 ms</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="H19" s="16" t="inlineStr">
         <is>
-          <t>38 ms</t>
+          <t>2938 ms</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="H20" s="18" t="inlineStr">
         <is>
-          <t>33 ms</t>
+          <t>2993 ms</t>
         </is>
       </c>
     </row>
@@ -1091,7 +1091,7 @@
       </c>
       <c r="H21" s="16" t="inlineStr">
         <is>
-          <t>32 ms</t>
+          <t>2816 ms</t>
         </is>
       </c>
     </row>
@@ -1120,7 +1120,7 @@
       </c>
       <c r="H22" s="18" t="inlineStr">
         <is>
-          <t>61 ms</t>
+          <t>2458 ms</t>
         </is>
       </c>
     </row>
@@ -1149,7 +1149,7 @@
       </c>
       <c r="H23" s="16" t="inlineStr">
         <is>
-          <t>24 ms</t>
+          <t>2722 ms</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1178,7 @@
       </c>
       <c r="H24" s="18" t="inlineStr">
         <is>
-          <t>31 ms</t>
+          <t>2451 ms</t>
         </is>
       </c>
     </row>
@@ -1207,7 +1207,7 @@
       </c>
       <c r="H25" s="16" t="inlineStr">
         <is>
-          <t>18 ms</t>
+          <t>20 ms</t>
         </is>
       </c>
     </row>
@@ -1250,7 +1250,7 @@
       </c>
       <c r="C30" s="21" t="inlineStr">
         <is>
-          <t>419 chars</t>
+          <t>1321 chars</t>
         </is>
       </c>
       <c r="D30" s="22" t="inlineStr">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="C31" s="21" t="inlineStr">
         <is>
-          <t>208 words</t>
+          <t>351 words</t>
         </is>
       </c>
       <c r="D31" s="22" t="inlineStr">
@@ -1557,17 +1557,17 @@
       </c>
       <c r="I2" s="27" t="inlineStr">
         <is>
-          <t>119 ms</t>
+          <t>3453 ms</t>
         </is>
       </c>
       <c r="J2" s="27" t="n">
-        <v>271</v>
+        <v>1207</v>
       </c>
       <c r="K2" s="18" t="n">
         <v>2</v>
       </c>
       <c r="L2" s="27" t="n">
-        <v>85</v>
+        <v>241</v>
       </c>
       <c r="M2" s="18" t="inlineStr">
         <is>
@@ -1581,15 +1581,15 @@
       </c>
       <c r="O2" s="18" t="inlineStr">
         <is>
-          <t>2.5 Hours Saved</t>
+          <t>2.3 Hours Saved</t>
         </is>
       </c>
       <c r="P2" s="18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q2" s="25" t="inlineStr">
         <is>
-          <t>High Quality: 2 chapters (85 words), 2 characters, 271 char gist</t>
+          <t>High Quality: 2 chapters (241 words), 2 characters, 1207 char gist</t>
         </is>
       </c>
     </row>
@@ -1634,17 +1634,17 @@
       </c>
       <c r="I3" s="29" t="inlineStr">
         <is>
-          <t>39 ms</t>
+          <t>3242 ms</t>
         </is>
       </c>
       <c r="J3" s="29" t="n">
-        <v>270</v>
+        <v>1204</v>
       </c>
       <c r="K3" s="16" t="n">
         <v>2</v>
       </c>
       <c r="L3" s="29" t="n">
-        <v>85</v>
+        <v>241</v>
       </c>
       <c r="M3" s="16" t="inlineStr">
         <is>
@@ -1658,15 +1658,15 @@
       </c>
       <c r="O3" s="16" t="inlineStr">
         <is>
-          <t>2.5 Hours Saved</t>
+          <t>2.3 Hours Saved</t>
         </is>
       </c>
       <c r="P3" s="16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q3" s="28" t="inlineStr">
         <is>
-          <t>High Quality: 2 chapters (85 words), 2 characters, 270 char gist</t>
+          <t>High Quality: 2 chapters (241 words), 2 characters, 1204 char gist</t>
         </is>
       </c>
     </row>
@@ -1711,17 +1711,17 @@
       </c>
       <c r="I4" s="27" t="inlineStr">
         <is>
-          <t>37 ms</t>
+          <t>3298 ms</t>
         </is>
       </c>
       <c r="J4" s="27" t="n">
-        <v>270</v>
+        <v>1204</v>
       </c>
       <c r="K4" s="18" t="n">
         <v>2</v>
       </c>
       <c r="L4" s="27" t="n">
-        <v>85</v>
+        <v>241</v>
       </c>
       <c r="M4" s="18" t="inlineStr">
         <is>
@@ -1735,15 +1735,15 @@
       </c>
       <c r="O4" s="18" t="inlineStr">
         <is>
-          <t>2.5 Hours Saved</t>
+          <t>2.3 Hours Saved</t>
         </is>
       </c>
       <c r="P4" s="18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q4" s="25" t="inlineStr">
         <is>
-          <t>High Quality: 2 chapters (85 words), 2 characters, 270 char gist</t>
+          <t>High Quality: 2 chapters (241 words), 2 characters, 1204 char gist</t>
         </is>
       </c>
     </row>
@@ -1788,17 +1788,17 @@
       </c>
       <c r="I5" s="29" t="inlineStr">
         <is>
-          <t>35 ms</t>
+          <t>2437 ms</t>
         </is>
       </c>
       <c r="J5" s="29" t="n">
-        <v>409</v>
+        <v>1340</v>
       </c>
       <c r="K5" s="16" t="n">
         <v>2</v>
       </c>
       <c r="L5" s="29" t="n">
-        <v>82</v>
+        <v>237</v>
       </c>
       <c r="M5" s="16" t="inlineStr">
         <is>
@@ -1812,15 +1812,15 @@
       </c>
       <c r="O5" s="16" t="inlineStr">
         <is>
-          <t>5.2 Hours Saved</t>
+          <t>9 Hours Saved</t>
         </is>
       </c>
       <c r="P5" s="16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q5" s="28" t="inlineStr">
         <is>
-          <t>High Quality: 2 chapters (82 words), 2 characters, 409 char gist</t>
+          <t>High Quality: 2 chapters (237 words), 2 characters, 1340 char gist</t>
         </is>
       </c>
     </row>
@@ -1865,17 +1865,17 @@
       </c>
       <c r="I6" s="27" t="inlineStr">
         <is>
-          <t>47 ms</t>
+          <t>3248 ms</t>
         </is>
       </c>
       <c r="J6" s="27" t="n">
-        <v>419</v>
+        <v>1372</v>
       </c>
       <c r="K6" s="18" t="n">
         <v>2</v>
       </c>
       <c r="L6" s="27" t="n">
-        <v>85</v>
+        <v>243</v>
       </c>
       <c r="M6" s="18" t="inlineStr">
         <is>
@@ -1889,15 +1889,15 @@
       </c>
       <c r="O6" s="18" t="inlineStr">
         <is>
-          <t>5.2 Hours Saved</t>
+          <t>4.8 Hours Saved</t>
         </is>
       </c>
       <c r="P6" s="18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q6" s="25" t="inlineStr">
         <is>
-          <t>High Quality: 2 chapters (85 words), 2 characters, 419 char gist</t>
+          <t>High Quality: 2 chapters (243 words), 2 characters, 1372 char gist</t>
         </is>
       </c>
     </row>
@@ -1942,17 +1942,17 @@
       </c>
       <c r="I7" s="29" t="inlineStr">
         <is>
-          <t>35 ms</t>
+          <t>2442 ms</t>
         </is>
       </c>
       <c r="J7" s="29" t="n">
-        <v>419</v>
+        <v>1360</v>
       </c>
       <c r="K7" s="16" t="n">
         <v>2</v>
       </c>
       <c r="L7" s="29" t="n">
-        <v>85</v>
+        <v>242</v>
       </c>
       <c r="M7" s="16" t="inlineStr">
         <is>
@@ -1966,15 +1966,15 @@
       </c>
       <c r="O7" s="16" t="inlineStr">
         <is>
-          <t>5.2 Hours Saved</t>
+          <t>9 Hours Saved</t>
         </is>
       </c>
       <c r="P7" s="16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q7" s="28" t="inlineStr">
         <is>
-          <t>High Quality: 2 chapters (85 words), 2 characters, 419 char gist</t>
+          <t>High Quality: 2 chapters (242 words), 2 characters, 1360 char gist</t>
         </is>
       </c>
     </row>
@@ -2019,17 +2019,17 @@
       </c>
       <c r="I8" s="27" t="inlineStr">
         <is>
-          <t>36 ms</t>
+          <t>3264 ms</t>
         </is>
       </c>
       <c r="J8" s="27" t="n">
-        <v>268</v>
+        <v>1198</v>
       </c>
       <c r="K8" s="18" t="n">
         <v>2</v>
       </c>
       <c r="L8" s="27" t="n">
-        <v>85</v>
+        <v>241</v>
       </c>
       <c r="M8" s="18" t="inlineStr">
         <is>
@@ -2043,15 +2043,15 @@
       </c>
       <c r="O8" s="18" t="inlineStr">
         <is>
-          <t>2.5 Hours Saved</t>
+          <t>2.3 Hours Saved</t>
         </is>
       </c>
       <c r="P8" s="18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q8" s="25" t="inlineStr">
         <is>
-          <t>High Quality: 2 chapters (85 words), 2 characters, 268 char gist</t>
+          <t>High Quality: 2 chapters (241 words), 2 characters, 1198 char gist</t>
         </is>
       </c>
     </row>
@@ -2096,11 +2096,11 @@
       </c>
       <c r="I9" s="29" t="inlineStr">
         <is>
-          <t>37 ms</t>
+          <t>3271 ms</t>
         </is>
       </c>
       <c r="J9" s="29" t="n">
-        <v>956</v>
+        <v>1434</v>
       </c>
       <c r="K9" s="16" t="n">
         <v>5</v>
@@ -2120,15 +2120,15 @@
       </c>
       <c r="O9" s="16" t="inlineStr">
         <is>
-          <t>15+ Hours Saved</t>
+          <t>4.7 Hours Saved</t>
         </is>
       </c>
       <c r="P9" s="16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q9" s="28" t="inlineStr">
         <is>
-          <t>High Quality: 5 chapters (1517 words), 6 characters, 956 char gist</t>
+          <t>High Quality: 5 chapters (1517 words), 6 characters, 1434 char gist</t>
         </is>
       </c>
     </row>
@@ -2173,11 +2173,11 @@
       </c>
       <c r="I10" s="27" t="inlineStr">
         <is>
-          <t>37 ms</t>
+          <t>3246 ms</t>
         </is>
       </c>
       <c r="J10" s="27" t="n">
-        <v>956</v>
+        <v>1434</v>
       </c>
       <c r="K10" s="18" t="n">
         <v>5</v>
@@ -2197,15 +2197,15 @@
       </c>
       <c r="O10" s="18" t="inlineStr">
         <is>
-          <t>15+ Hours Saved</t>
+          <t>4.7 Hours Saved</t>
         </is>
       </c>
       <c r="P10" s="18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q10" s="25" t="inlineStr">
         <is>
-          <t>High Quality: 5 chapters (1517 words), 6 characters, 956 char gist</t>
+          <t>High Quality: 5 chapters (1517 words), 6 characters, 1434 char gist</t>
         </is>
       </c>
     </row>
@@ -2250,11 +2250,11 @@
       </c>
       <c r="I11" s="29" t="inlineStr">
         <is>
-          <t>29 ms</t>
+          <t>3267 ms</t>
         </is>
       </c>
       <c r="J11" s="29" t="n">
-        <v>957</v>
+        <v>1435</v>
       </c>
       <c r="K11" s="16" t="n">
         <v>5</v>
@@ -2274,15 +2274,15 @@
       </c>
       <c r="O11" s="16" t="inlineStr">
         <is>
-          <t>15+ Hours Saved</t>
+          <t>4.7 Hours Saved</t>
         </is>
       </c>
       <c r="P11" s="16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q11" s="28" t="inlineStr">
         <is>
-          <t>High Quality: 5 chapters (1517 words), 6 characters, 957 char gist</t>
+          <t>High Quality: 5 chapters (1517 words), 6 characters, 1435 char gist</t>
         </is>
       </c>
     </row>
@@ -2327,17 +2327,17 @@
       </c>
       <c r="I12" s="27" t="inlineStr">
         <is>
-          <t>32 ms</t>
+          <t>3254 ms</t>
         </is>
       </c>
       <c r="J12" s="27" t="n">
-        <v>273</v>
+        <v>1213</v>
       </c>
       <c r="K12" s="18" t="n">
         <v>2</v>
       </c>
       <c r="L12" s="27" t="n">
-        <v>88</v>
+        <v>246</v>
       </c>
       <c r="M12" s="18" t="inlineStr">
         <is>
@@ -2351,15 +2351,15 @@
       </c>
       <c r="O12" s="18" t="inlineStr">
         <is>
-          <t>2.5 Hours Saved</t>
+          <t>2.3 Hours Saved</t>
         </is>
       </c>
       <c r="P12" s="18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q12" s="25" t="inlineStr">
         <is>
-          <t>High Quality: 2 chapters (88 words), 2 characters, 273 char gist</t>
+          <t>High Quality: 2 chapters (246 words), 2 characters, 1213 char gist</t>
         </is>
       </c>
     </row>
@@ -2404,17 +2404,17 @@
       </c>
       <c r="I13" s="29" t="inlineStr">
         <is>
-          <t>29 ms</t>
+          <t>2459 ms</t>
         </is>
       </c>
       <c r="J13" s="29" t="n">
-        <v>419</v>
+        <v>1360</v>
       </c>
       <c r="K13" s="16" t="n">
         <v>2</v>
       </c>
       <c r="L13" s="29" t="n">
-        <v>85</v>
+        <v>242</v>
       </c>
       <c r="M13" s="16" t="inlineStr">
         <is>
@@ -2428,15 +2428,15 @@
       </c>
       <c r="O13" s="16" t="inlineStr">
         <is>
-          <t>5.2 Hours Saved</t>
+          <t>9 Hours Saved</t>
         </is>
       </c>
       <c r="P13" s="16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q13" s="28" t="inlineStr">
         <is>
-          <t>High Quality: 2 chapters (85 words), 2 characters, 419 char gist</t>
+          <t>High Quality: 2 chapters (242 words), 2 characters, 1360 char gist</t>
         </is>
       </c>
     </row>
@@ -2481,17 +2481,17 @@
       </c>
       <c r="I14" s="27" t="inlineStr">
         <is>
-          <t>33 ms</t>
+          <t>2460 ms</t>
         </is>
       </c>
       <c r="J14" s="27" t="n">
-        <v>420</v>
+        <v>1361</v>
       </c>
       <c r="K14" s="18" t="n">
         <v>2</v>
       </c>
       <c r="L14" s="27" t="n">
-        <v>85</v>
+        <v>242</v>
       </c>
       <c r="M14" s="18" t="inlineStr">
         <is>
@@ -2505,15 +2505,15 @@
       </c>
       <c r="O14" s="18" t="inlineStr">
         <is>
-          <t>5.2 Hours Saved</t>
+          <t>9 Hours Saved</t>
         </is>
       </c>
       <c r="P14" s="18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q14" s="25" t="inlineStr">
         <is>
-          <t>High Quality: 2 chapters (85 words), 2 characters, 420 char gist</t>
+          <t>High Quality: 2 chapters (242 words), 2 characters, 1361 char gist</t>
         </is>
       </c>
     </row>
@@ -2558,17 +2558,17 @@
       </c>
       <c r="I15" s="29" t="inlineStr">
         <is>
-          <t>36 ms</t>
+          <t>3267 ms</t>
         </is>
       </c>
       <c r="J15" s="29" t="n">
-        <v>267</v>
+        <v>1195</v>
       </c>
       <c r="K15" s="16" t="n">
         <v>2</v>
       </c>
       <c r="L15" s="29" t="n">
-        <v>82</v>
+        <v>236</v>
       </c>
       <c r="M15" s="16" t="inlineStr">
         <is>
@@ -2582,15 +2582,15 @@
       </c>
       <c r="O15" s="16" t="inlineStr">
         <is>
-          <t>2.5 Hours Saved</t>
+          <t>2.3 Hours Saved</t>
         </is>
       </c>
       <c r="P15" s="16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q15" s="28" t="inlineStr">
         <is>
-          <t>High Quality: 2 chapters (82 words), 2 characters, 267 char gist</t>
+          <t>High Quality: 2 chapters (236 words), 2 characters, 1195 char gist</t>
         </is>
       </c>
     </row>
@@ -2635,17 +2635,17 @@
       </c>
       <c r="I16" s="27" t="inlineStr">
         <is>
-          <t>35 ms</t>
+          <t>2458 ms</t>
         </is>
       </c>
       <c r="J16" s="27" t="n">
-        <v>425</v>
+        <v>1372</v>
       </c>
       <c r="K16" s="18" t="n">
         <v>2</v>
       </c>
       <c r="L16" s="27" t="n">
-        <v>88</v>
+        <v>247</v>
       </c>
       <c r="M16" s="18" t="inlineStr">
         <is>
@@ -2659,15 +2659,15 @@
       </c>
       <c r="O16" s="18" t="inlineStr">
         <is>
-          <t>5.2 Hours Saved</t>
+          <t>9 Hours Saved</t>
         </is>
       </c>
       <c r="P16" s="18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q16" s="25" t="inlineStr">
         <is>
-          <t>High Quality: 2 chapters (88 words), 2 characters, 425 char gist</t>
+          <t>High Quality: 2 chapters (247 words), 2 characters, 1372 char gist</t>
         </is>
       </c>
     </row>
@@ -2712,17 +2712,17 @@
       </c>
       <c r="I17" s="29" t="inlineStr">
         <is>
-          <t>32 ms</t>
+          <t>3260 ms</t>
         </is>
       </c>
       <c r="J17" s="29" t="n">
-        <v>425</v>
+        <v>1384</v>
       </c>
       <c r="K17" s="16" t="n">
         <v>2</v>
       </c>
       <c r="L17" s="29" t="n">
-        <v>88</v>
+        <v>248</v>
       </c>
       <c r="M17" s="16" t="inlineStr">
         <is>
@@ -2736,15 +2736,15 @@
       </c>
       <c r="O17" s="16" t="inlineStr">
         <is>
-          <t>5.2 Hours Saved</t>
+          <t>4.8 Hours Saved</t>
         </is>
       </c>
       <c r="P17" s="16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q17" s="28" t="inlineStr">
         <is>
-          <t>High Quality: 2 chapters (88 words), 2 characters, 425 char gist</t>
+          <t>High Quality: 2 chapters (248 words), 2 characters, 1384 char gist</t>
         </is>
       </c>
     </row>
@@ -2789,17 +2789,17 @@
       </c>
       <c r="I18" s="27" t="inlineStr">
         <is>
-          <t>40 ms</t>
+          <t>3272 ms</t>
         </is>
       </c>
       <c r="J18" s="27" t="n">
-        <v>426</v>
+        <v>1385</v>
       </c>
       <c r="K18" s="18" t="n">
         <v>2</v>
       </c>
       <c r="L18" s="27" t="n">
-        <v>88</v>
+        <v>248</v>
       </c>
       <c r="M18" s="18" t="inlineStr">
         <is>
@@ -2813,15 +2813,15 @@
       </c>
       <c r="O18" s="18" t="inlineStr">
         <is>
-          <t>5.2 Hours Saved</t>
+          <t>4.8 Hours Saved</t>
         </is>
       </c>
       <c r="P18" s="18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q18" s="25" t="inlineStr">
         <is>
-          <t>High Quality: 2 chapters (88 words), 2 characters, 426 char gist</t>
+          <t>High Quality: 2 chapters (248 words), 2 characters, 1385 char gist</t>
         </is>
       </c>
     </row>
@@ -2866,17 +2866,17 @@
       </c>
       <c r="I19" s="29" t="inlineStr">
         <is>
-          <t>28 ms</t>
+          <t>3270 ms</t>
         </is>
       </c>
       <c r="J19" s="29" t="n">
-        <v>270</v>
+        <v>1204</v>
       </c>
       <c r="K19" s="16" t="n">
         <v>2</v>
       </c>
       <c r="L19" s="29" t="n">
-        <v>82</v>
+        <v>236</v>
       </c>
       <c r="M19" s="16" t="inlineStr">
         <is>
@@ -2890,15 +2890,15 @@
       </c>
       <c r="O19" s="16" t="inlineStr">
         <is>
-          <t>2.5 Hours Saved</t>
+          <t>2.3 Hours Saved</t>
         </is>
       </c>
       <c r="P19" s="16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q19" s="28" t="inlineStr">
         <is>
-          <t>High Quality: 2 chapters (82 words), 2 characters, 270 char gist</t>
+          <t>High Quality: 2 chapters (236 words), 2 characters, 1204 char gist</t>
         </is>
       </c>
     </row>
@@ -2943,17 +2943,17 @@
       </c>
       <c r="I20" s="27" t="inlineStr">
         <is>
-          <t>28 ms</t>
+          <t>2455 ms</t>
         </is>
       </c>
       <c r="J20" s="27" t="n">
-        <v>425</v>
+        <v>1372</v>
       </c>
       <c r="K20" s="18" t="n">
         <v>2</v>
       </c>
       <c r="L20" s="27" t="n">
-        <v>85</v>
+        <v>242</v>
       </c>
       <c r="M20" s="18" t="inlineStr">
         <is>
@@ -2967,15 +2967,15 @@
       </c>
       <c r="O20" s="18" t="inlineStr">
         <is>
-          <t>5.2 Hours Saved</t>
+          <t>9 Hours Saved</t>
         </is>
       </c>
       <c r="P20" s="18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q20" s="25" t="inlineStr">
         <is>
-          <t>High Quality: 2 chapters (85 words), 2 characters, 425 char gist</t>
+          <t>High Quality: 2 chapters (242 words), 2 characters, 1372 char gist</t>
         </is>
       </c>
     </row>
@@ -3020,17 +3020,17 @@
       </c>
       <c r="I21" s="29" t="inlineStr">
         <is>
-          <t>34 ms</t>
+          <t>2447 ms</t>
         </is>
       </c>
       <c r="J21" s="29" t="n">
-        <v>425</v>
+        <v>1372</v>
       </c>
       <c r="K21" s="16" t="n">
         <v>2</v>
       </c>
       <c r="L21" s="29" t="n">
-        <v>85</v>
+        <v>242</v>
       </c>
       <c r="M21" s="16" t="inlineStr">
         <is>
@@ -3044,15 +3044,15 @@
       </c>
       <c r="O21" s="16" t="inlineStr">
         <is>
-          <t>5.2 Hours Saved</t>
+          <t>9 Hours Saved</t>
         </is>
       </c>
       <c r="P21" s="16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q21" s="28" t="inlineStr">
         <is>
-          <t>High Quality: 2 chapters (85 words), 2 characters, 425 char gist</t>
+          <t>High Quality: 2 chapters (242 words), 2 characters, 1372 char gist</t>
         </is>
       </c>
     </row>
@@ -3097,17 +3097,17 @@
       </c>
       <c r="I22" s="27" t="inlineStr">
         <is>
-          <t>61 ms</t>
+          <t>2458 ms</t>
         </is>
       </c>
       <c r="J22" s="27" t="n">
-        <v>411</v>
+        <v>1344</v>
       </c>
       <c r="K22" s="18" t="n">
         <v>2</v>
       </c>
       <c r="L22" s="27" t="n">
-        <v>82</v>
+        <v>237</v>
       </c>
       <c r="M22" s="18" t="inlineStr">
         <is>
@@ -3121,15 +3121,15 @@
       </c>
       <c r="O22" s="18" t="inlineStr">
         <is>
-          <t>5.2 Hours Saved</t>
+          <t>9 Hours Saved</t>
         </is>
       </c>
       <c r="P22" s="18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q22" s="25" t="inlineStr">
         <is>
-          <t>High Quality: 2 chapters (82 words), 2 characters, 411 char gist</t>
+          <t>High Quality: 2 chapters (237 words), 2 characters, 1344 char gist</t>
         </is>
       </c>
     </row>
@@ -3174,17 +3174,17 @@
       </c>
       <c r="I23" s="29" t="inlineStr">
         <is>
-          <t>24 ms</t>
+          <t>2456 ms</t>
         </is>
       </c>
       <c r="J23" s="29" t="n">
-        <v>411</v>
+        <v>1344</v>
       </c>
       <c r="K23" s="16" t="n">
         <v>2</v>
       </c>
       <c r="L23" s="29" t="n">
-        <v>85</v>
+        <v>242</v>
       </c>
       <c r="M23" s="16" t="inlineStr">
         <is>
@@ -3198,15 +3198,15 @@
       </c>
       <c r="O23" s="16" t="inlineStr">
         <is>
-          <t>5.2 Hours Saved</t>
+          <t>9 Hours Saved</t>
         </is>
       </c>
       <c r="P23" s="16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q23" s="28" t="inlineStr">
         <is>
-          <t>High Quality: 2 chapters (85 words), 2 characters, 411 char gist</t>
+          <t>High Quality: 2 chapters (242 words), 2 characters, 1344 char gist</t>
         </is>
       </c>
     </row>
@@ -3251,17 +3251,17 @@
       </c>
       <c r="I24" s="27" t="inlineStr">
         <is>
-          <t>29 ms</t>
+          <t>2459 ms</t>
         </is>
       </c>
       <c r="J24" s="27" t="n">
-        <v>411</v>
+        <v>1344</v>
       </c>
       <c r="K24" s="18" t="n">
         <v>2</v>
       </c>
       <c r="L24" s="27" t="n">
-        <v>85</v>
+        <v>242</v>
       </c>
       <c r="M24" s="18" t="inlineStr">
         <is>
@@ -3275,15 +3275,15 @@
       </c>
       <c r="O24" s="18" t="inlineStr">
         <is>
-          <t>5.2 Hours Saved</t>
+          <t>9 Hours Saved</t>
         </is>
       </c>
       <c r="P24" s="18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q24" s="25" t="inlineStr">
         <is>
-          <t>High Quality: 2 chapters (85 words), 2 characters, 411 char gist</t>
+          <t>High Quality: 2 chapters (242 words), 2 characters, 1344 char gist</t>
         </is>
       </c>
     </row>
@@ -3328,17 +3328,17 @@
       </c>
       <c r="I25" s="29" t="inlineStr">
         <is>
-          <t>25 ms</t>
+          <t>2457 ms</t>
         </is>
       </c>
       <c r="J25" s="29" t="n">
-        <v>415</v>
+        <v>1352</v>
       </c>
       <c r="K25" s="16" t="n">
         <v>2</v>
       </c>
       <c r="L25" s="29" t="n">
-        <v>85</v>
+        <v>242</v>
       </c>
       <c r="M25" s="16" t="inlineStr">
         <is>
@@ -3352,15 +3352,15 @@
       </c>
       <c r="O25" s="16" t="inlineStr">
         <is>
-          <t>5.2 Hours Saved</t>
+          <t>9 Hours Saved</t>
         </is>
       </c>
       <c r="P25" s="16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q25" s="28" t="inlineStr">
         <is>
-          <t>High Quality: 2 chapters (85 words), 2 characters, 415 char gist</t>
+          <t>High Quality: 2 chapters (242 words), 2 characters, 1352 char gist</t>
         </is>
       </c>
     </row>
@@ -3405,17 +3405,17 @@
       </c>
       <c r="I26" s="27" t="inlineStr">
         <is>
-          <t>31 ms</t>
+          <t>2451 ms</t>
         </is>
       </c>
       <c r="J26" s="27" t="n">
-        <v>413</v>
+        <v>1348</v>
       </c>
       <c r="K26" s="18" t="n">
         <v>2</v>
       </c>
       <c r="L26" s="27" t="n">
-        <v>82</v>
+        <v>237</v>
       </c>
       <c r="M26" s="18" t="inlineStr">
         <is>
@@ -3429,15 +3429,15 @@
       </c>
       <c r="O26" s="18" t="inlineStr">
         <is>
-          <t>5.2 Hours Saved</t>
+          <t>9 Hours Saved</t>
         </is>
       </c>
       <c r="P26" s="18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q26" s="25" t="inlineStr">
         <is>
-          <t>High Quality: 2 chapters (82 words), 2 characters, 413 char gist</t>
+          <t>High Quality: 2 chapters (237 words), 2 characters, 1348 char gist</t>
         </is>
       </c>
     </row>
@@ -3482,17 +3482,17 @@
       </c>
       <c r="I27" s="29" t="inlineStr">
         <is>
-          <t>31 ms</t>
+          <t>3263 ms</t>
         </is>
       </c>
       <c r="J27" s="29" t="n">
-        <v>261</v>
+        <v>1177</v>
       </c>
       <c r="K27" s="16" t="n">
         <v>2</v>
       </c>
       <c r="L27" s="29" t="n">
-        <v>82</v>
+        <v>236</v>
       </c>
       <c r="M27" s="16" t="inlineStr">
         <is>
@@ -3506,15 +3506,15 @@
       </c>
       <c r="O27" s="16" t="inlineStr">
         <is>
-          <t>2.5 Hours Saved</t>
+          <t>2.3 Hours Saved</t>
         </is>
       </c>
       <c r="P27" s="16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q27" s="28" t="inlineStr">
         <is>
-          <t>High Quality: 2 chapters (82 words), 2 characters, 261 char gist</t>
+          <t>High Quality: 2 chapters (236 words), 2 characters, 1177 char gist</t>
         </is>
       </c>
     </row>
@@ -3559,17 +3559,17 @@
       </c>
       <c r="I28" s="27" t="inlineStr">
         <is>
-          <t>23 ms</t>
+          <t>2445 ms</t>
         </is>
       </c>
       <c r="J28" s="27" t="n">
-        <v>433</v>
+        <v>1388</v>
       </c>
       <c r="K28" s="18" t="n">
         <v>2</v>
       </c>
       <c r="L28" s="27" t="n">
-        <v>91</v>
+        <v>252</v>
       </c>
       <c r="M28" s="18" t="inlineStr">
         <is>
@@ -3583,15 +3583,15 @@
       </c>
       <c r="O28" s="18" t="inlineStr">
         <is>
-          <t>5.2 Hours Saved</t>
+          <t>9 Hours Saved</t>
         </is>
       </c>
       <c r="P28" s="18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q28" s="25" t="inlineStr">
         <is>
-          <t>High Quality: 2 chapters (91 words), 2 characters, 433 char gist</t>
+          <t>High Quality: 2 chapters (252 words), 2 characters, 1388 char gist</t>
         </is>
       </c>
     </row>
@@ -3636,17 +3636,17 @@
       </c>
       <c r="I29" s="29" t="inlineStr">
         <is>
-          <t>18 ms</t>
+          <t>3265 ms</t>
         </is>
       </c>
       <c r="J29" s="29" t="n">
-        <v>269</v>
+        <v>1201</v>
       </c>
       <c r="K29" s="16" t="n">
         <v>2</v>
       </c>
       <c r="L29" s="29" t="n">
-        <v>82</v>
+        <v>236</v>
       </c>
       <c r="M29" s="16" t="inlineStr">
         <is>
@@ -3660,15 +3660,15 @@
       </c>
       <c r="O29" s="16" t="inlineStr">
         <is>
-          <t>2.5 Hours Saved</t>
+          <t>2.3 Hours Saved</t>
         </is>
       </c>
       <c r="P29" s="16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q29" s="28" t="inlineStr">
         <is>
-          <t>High Quality: 2 chapters (82 words), 2 characters, 269 char gist</t>
+          <t>High Quality: 2 chapters (236 words), 2 characters, 1201 char gist</t>
         </is>
       </c>
     </row>
@@ -3713,17 +3713,17 @@
       </c>
       <c r="I30" s="27" t="inlineStr">
         <is>
-          <t>23 ms</t>
+          <t>2449 ms</t>
         </is>
       </c>
       <c r="J30" s="27" t="n">
-        <v>409</v>
+        <v>1340</v>
       </c>
       <c r="K30" s="18" t="n">
         <v>2</v>
       </c>
       <c r="L30" s="27" t="n">
-        <v>82</v>
+        <v>237</v>
       </c>
       <c r="M30" s="18" t="inlineStr">
         <is>
@@ -3737,15 +3737,15 @@
       </c>
       <c r="O30" s="18" t="inlineStr">
         <is>
-          <t>5.2 Hours Saved</t>
+          <t>9 Hours Saved</t>
         </is>
       </c>
       <c r="P30" s="18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q30" s="25" t="inlineStr">
         <is>
-          <t>High Quality: 2 chapters (82 words), 2 characters, 409 char gist</t>
+          <t>High Quality: 2 chapters (237 words), 2 characters, 1340 char gist</t>
         </is>
       </c>
     </row>
@@ -3790,17 +3790,17 @@
       </c>
       <c r="I31" s="29" t="inlineStr">
         <is>
-          <t>24 ms</t>
+          <t>2454 ms</t>
         </is>
       </c>
       <c r="J31" s="29" t="n">
-        <v>407</v>
+        <v>1336</v>
       </c>
       <c r="K31" s="16" t="n">
         <v>2</v>
       </c>
       <c r="L31" s="29" t="n">
-        <v>82</v>
+        <v>237</v>
       </c>
       <c r="M31" s="16" t="inlineStr">
         <is>
@@ -3814,15 +3814,15 @@
       </c>
       <c r="O31" s="16" t="inlineStr">
         <is>
-          <t>5.2 Hours Saved</t>
+          <t>9 Hours Saved</t>
         </is>
       </c>
       <c r="P31" s="16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q31" s="28" t="inlineStr">
         <is>
-          <t>High Quality: 2 chapters (82 words), 2 characters, 407 char gist</t>
+          <t>High Quality: 2 chapters (237 words), 2 characters, 1336 char gist</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
       </c>
       <c r="I32" s="27" t="inlineStr">
         <is>
-          <t>35 ms</t>
+          <t>36 ms</t>
         </is>
       </c>
       <c r="J32" s="27" t="inlineStr">
@@ -3956,7 +3956,7 @@
       </c>
       <c r="I33" s="29" t="inlineStr">
         <is>
-          <t>16 ms</t>
+          <t>20 ms</t>
         </is>
       </c>
       <c r="J33" s="29" t="inlineStr">
@@ -4043,7 +4043,7 @@
       </c>
       <c r="I34" s="27" t="inlineStr">
         <is>
-          <t>10 ms</t>
+          <t>18 ms</t>
         </is>
       </c>
       <c r="J34" s="27" t="inlineStr">
@@ -4130,7 +4130,7 @@
       </c>
       <c r="I35" s="29" t="inlineStr">
         <is>
-          <t>22 ms</t>
+          <t>19 ms</t>
         </is>
       </c>
       <c r="J35" s="29" t="inlineStr">
@@ -4217,7 +4217,7 @@
       </c>
       <c r="I36" s="27" t="inlineStr">
         <is>
-          <t>5 ms</t>
+          <t>6 ms</t>
         </is>
       </c>
       <c r="J36" s="27" t="inlineStr">
@@ -4391,7 +4391,7 @@
       </c>
       <c r="I38" s="27" t="inlineStr">
         <is>
-          <t>7 ms</t>
+          <t>3 ms</t>
         </is>
       </c>
       <c r="J38" s="27" t="inlineStr">
@@ -4478,17 +4478,17 @@
       </c>
       <c r="I39" s="29" t="inlineStr">
         <is>
-          <t>38 ms</t>
+          <t>3257 ms</t>
         </is>
       </c>
       <c r="J39" s="29" t="n">
-        <v>417</v>
+        <v>1368</v>
       </c>
       <c r="K39" s="16" t="n">
         <v>2</v>
       </c>
       <c r="L39" s="29" t="n">
-        <v>82</v>
+        <v>238</v>
       </c>
       <c r="M39" s="16" t="inlineStr">
         <is>
@@ -4502,15 +4502,15 @@
       </c>
       <c r="O39" s="16" t="inlineStr">
         <is>
-          <t>5.2 Hours Saved</t>
+          <t>4.8 Hours Saved</t>
         </is>
       </c>
       <c r="P39" s="16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q39" s="28" t="inlineStr">
         <is>
-          <t>High Quality: 2 chapters (82 words), 2 characters, 417 char gist</t>
+          <t>High Quality: 2 chapters (238 words), 2 characters, 1368 char gist</t>
         </is>
       </c>
     </row>
@@ -4557,17 +4557,17 @@
       </c>
       <c r="I40" s="27" t="inlineStr">
         <is>
-          <t>23 ms</t>
+          <t>3268 ms</t>
         </is>
       </c>
       <c r="J40" s="27" t="n">
-        <v>293</v>
+        <v>1273</v>
       </c>
       <c r="K40" s="18" t="n">
         <v>2</v>
       </c>
       <c r="L40" s="27" t="n">
-        <v>91</v>
+        <v>251</v>
       </c>
       <c r="M40" s="18" t="inlineStr">
         <is>
@@ -4581,15 +4581,15 @@
       </c>
       <c r="O40" s="18" t="inlineStr">
         <is>
-          <t>2.5 Hours Saved</t>
+          <t>2.3 Hours Saved</t>
         </is>
       </c>
       <c r="P40" s="18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q40" s="25" t="inlineStr">
         <is>
-          <t>High Quality: 2 chapters (91 words), 2 characters, 293 char gist</t>
+          <t>High Quality: 2 chapters (251 words), 2 characters, 1273 char gist</t>
         </is>
       </c>
     </row>
@@ -4636,17 +4636,17 @@
       </c>
       <c r="I41" s="29" t="inlineStr">
         <is>
-          <t>26 ms</t>
+          <t>3262 ms</t>
         </is>
       </c>
       <c r="J41" s="29" t="n">
-        <v>273</v>
+        <v>1213</v>
       </c>
       <c r="K41" s="16" t="n">
         <v>2</v>
       </c>
       <c r="L41" s="29" t="n">
-        <v>88</v>
+        <v>246</v>
       </c>
       <c r="M41" s="16" t="inlineStr">
         <is>
@@ -4660,15 +4660,15 @@
       </c>
       <c r="O41" s="16" t="inlineStr">
         <is>
-          <t>2.5 Hours Saved</t>
+          <t>2.3 Hours Saved</t>
         </is>
       </c>
       <c r="P41" s="16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q41" s="28" t="inlineStr">
         <is>
-          <t>High Quality: 2 chapters (88 words), 2 characters, 273 char gist</t>
+          <t>High Quality: 2 chapters (246 words), 2 characters, 1213 char gist</t>
         </is>
       </c>
     </row>
@@ -4715,17 +4715,17 @@
       </c>
       <c r="I42" s="27" t="inlineStr">
         <is>
-          <t>33 ms</t>
+          <t>2446 ms</t>
         </is>
       </c>
       <c r="J42" s="27" t="n">
-        <v>427</v>
+        <v>1374</v>
       </c>
       <c r="K42" s="18" t="n">
         <v>2</v>
       </c>
       <c r="L42" s="27" t="n">
-        <v>85</v>
+        <v>242</v>
       </c>
       <c r="M42" s="18" t="inlineStr">
         <is>
@@ -4739,15 +4739,15 @@
       </c>
       <c r="O42" s="18" t="inlineStr">
         <is>
-          <t>5.2 Hours Saved</t>
+          <t>9 Hours Saved</t>
         </is>
       </c>
       <c r="P42" s="18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q42" s="25" t="inlineStr">
         <is>
-          <t>High Quality: 2 chapters (85 words), 2 characters, 427 char gist</t>
+          <t>High Quality: 2 chapters (242 words), 2 characters, 1374 char gist</t>
         </is>
       </c>
     </row>
@@ -4794,17 +4794,17 @@
       </c>
       <c r="I43" s="29" t="inlineStr">
         <is>
-          <t>33 ms</t>
+          <t>2453 ms</t>
         </is>
       </c>
       <c r="J43" s="29" t="n">
-        <v>451</v>
+        <v>1424</v>
       </c>
       <c r="K43" s="16" t="n">
         <v>2</v>
       </c>
       <c r="L43" s="29" t="n">
-        <v>82</v>
+        <v>237</v>
       </c>
       <c r="M43" s="16" t="inlineStr">
         <is>
@@ -4818,15 +4818,15 @@
       </c>
       <c r="O43" s="16" t="inlineStr">
         <is>
-          <t>5.2 Hours Saved</t>
+          <t>9 Hours Saved</t>
         </is>
       </c>
       <c r="P43" s="16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q43" s="28" t="inlineStr">
         <is>
-          <t>High Quality: 2 chapters (82 words), 2 characters, 451 char gist</t>
+          <t>High Quality: 2 chapters (237 words), 2 characters, 1424 char gist</t>
         </is>
       </c>
     </row>

</xml_diff>